<commit_message>
feat(F-NAR-019): TREE-DIF-058 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-DIF-058.xlsx
+++ b/stories/arbres/TREE-DIF-058.xlsx
@@ -3280,17 +3280,17 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Sur le tabouret, deux têtes se calment. Nino, tu l'as vue glisser. Oui, tout près de tes mains. Toi haute, lui qui noue, ça tenait. Vos voix sont devenues toutes petites. Les clochettes restent dans la paume de Chouchou. Je reste un peu. Une poussière reste collée aux cheveux. Une poussière dore les cheveux, sous l'abat-jour.</t>
+          <t>Sur le tabouret, deux têtes se calment. Nino, tu l'as vue glisser. Oui, tout près de tes mains. Toi haute, lui qui noue, ça tenait. Vos voix sont devenues toutes petites. Les clochettes restent dans la paume de Chouchou. Je reste un peu. Tes cheveux sentent le bois. Une poussière dore les cheveux, sous l'abat-jour.</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Sur le tabouret, deux têtes se calment. Nino, tu l'as vue glisser. Oui, tout près de tes mains. Toi haute, lui qui noue, ça tenait. Vos voix sont devenues toutes petites. Les clochettes restent dans la paume de Chouchou. Je reste un peu. Une poussière reste collée aux cheveux. Une poussière dore les cheveux, sous l'abat-jour.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Sur le tabouret, deux têtes se calment. Nino, tu l'as vue glisser. Oui, tout près de tes mains. Toi haute, lui qui noue, ça tenait. Vos voix sont devenues toutes petites. Les clochettes restent dans la paume de Chouchou. Je reste un peu. Tes cheveux sentent le bois. Une poussière dore les cheveux, sous l'abat-jour.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Sur le tabouret, deux têtes se calment. Nino, tu l'as vue glisser. Oui, tout près de tes mains. Toi haute, lui qui noue, ça tenait. Vos voix sont devenues toutes petites. Les clochettes restent dans la paume de Chouchou. Je reste un peu. Une poussière reste collée aux cheveux. Une poussière dore les cheveux, sous l'abat-jour.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Sur le tabouret, deux têtes se calment. Nino, tu l'as vue glisser. Oui, tout près de tes mains. Toi haute, lui qui noue, ça tenait. Vos voix sont devenues toutes petites. Les clochettes restent dans la paume de Chouchou. Je reste un peu. Tes cheveux sentent le bois. Une poussière dore les cheveux, sous l'abat-jour.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr"/>
@@ -3435,7 +3435,7 @@
 maman|Vos voix sont devenues toutes petites.
 narrateur|Les clochettes restent dans la paume de Chouchou.
 copain|Je reste un peu.
-narrateur|Une poussière reste collée aux cheveux.
+enfant-f|Tes cheveux sentent le bois.
 narrateur|Une poussière dore les cheveux, sous l'abat-jour.</t>
         </is>
       </c>
@@ -5908,17 +5908,17 @@
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Les talons de Nino sont chauds. Tu as tenu le haut pour moi. Tu nouais le bas. Le carreau sent le soir, tout près. La porte sonnera, demain. Chouchou les pose contre la vitre. Les clochettes pèsent sur le loquet. Un rai jaune traverse le métal. Un rai jaune traverse le loquet.</t>
+          <t>Les talons de Nino sont chauds. Tu as tenu le haut pour moi. Tu nouais le bas. Le carreau sent le soir, tout près. La porte sonnera, demain. Je les pose contre la vitre. Les clochettes pèsent sur le loquet. Le jaune de la rue les touche. Un rai jaune traverse le loquet.</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les talons de Nino sont chauds. Tu as tenu le haut pour moi. Tu nouais le bas. Le carreau sent le soir, tout près. La porte sonnera, demain. Chouchou les pose contre la vitre. Les clochettes pèsent sur le loquet. Un rai jaune traverse le métal. Un rai jaune traverse le loquet.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les talons de Nino sont chauds. Tu as tenu le haut pour moi. Tu nouais le bas. Le carreau sent le soir, tout près. La porte sonnera, demain. Je les pose contre la vitre. Les clochettes pèsent sur le loquet. Le jaune de la rue les touche. Un rai jaune traverse le loquet.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les talons de Nino sont chauds. Tu as tenu le haut pour moi. Tu nouais le bas. Le carreau sent le soir, tout près. La porte sonnera, demain. Chouchou les pose contre la vitre. Les clochettes pèsent sur le loquet. Un rai jaune traverse le métal. Un rai jaune traverse le loquet.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les talons de Nino sont chauds. Tu as tenu le haut pour moi. Tu nouais le bas. Le carreau sent le soir, tout près. La porte sonnera, demain. Je les pose contre la vitre. Les clochettes pèsent sur le loquet. Le jaune de la rue les touche. Un rai jaune traverse le loquet.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr"/>
@@ -6061,9 +6061,9 @@
 copain|Tu nouais le bas.
 maman|Le carreau sent le soir, tout près.
 papa|La porte sonnera, demain.
-narrateur|Chouchou les pose contre la vitre.
+enfant-f|Je les pose contre la vitre.
 narrateur|Les clochettes pèsent sur le loquet.
-narrateur|Un rai jaune traverse le métal.
+copain|Le jaune de la rue les touche.
 narrateur|Un rai jaune traverse le loquet.</t>
         </is>
       </c>
@@ -8532,17 +8532,17 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Sur le tabouret, deux têtes se calment. Nino, tu l'as vue glisser. Oui, tout près de tes mains. Toi haute, lui qui noue, ça tenait. Vos voix sont devenues toutes petites. Le ruban reste dans la paume de Chouchou. Je reste un peu. Une poussière reste collée aux cheveux. Le tabouret garde une mèche, dans l'ombre jaune.</t>
+          <t>Sur le tabouret, deux têtes se calment. Nino, tu l'as vue glisser. Oui, tout près de tes mains. Toi haute, lui qui noue, ça tenait. Vos voix sont devenues toutes petites. Le ruban reste dans la paume de Chouchou. Je reste un peu. Une mèche à toi, sur le bois. Le tabouret garde une mèche, dans l'ombre jaune.</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Sur le tabouret, deux têtes se calment. Nino, tu l'as vue glisser. Oui, tout près de tes mains. Toi haute, lui qui noue, ça tenait. Vos voix sont devenues toutes petites. Le ruban reste dans la paume de Chouchou. Je reste un peu. Une poussière reste collée aux cheveux. Le tabouret garde une mèche, dans l'ombre jaune.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Sur le tabouret, deux têtes se calment. Nino, tu l'as vue glisser. Oui, tout près de tes mains. Toi haute, lui qui noue, ça tenait. Vos voix sont devenues toutes petites. Le ruban reste dans la paume de Chouchou. Je reste un peu. Une mèche à toi, sur le bois. Le tabouret garde une mèche, dans l'ombre jaune.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Sur le tabouret, deux têtes se calment. Nino, tu l'as vue glisser. Oui, tout près de tes mains. Toi haute, lui qui noue, ça tenait. Vos voix sont devenues toutes petites. Le ruban reste dans la paume de Chouchou. Je reste un peu. Une poussière reste collée aux cheveux. Le tabouret garde une mèche, dans l'ombre jaune.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Sur le tabouret, deux têtes se calment. Nino, tu l'as vue glisser. Oui, tout près de tes mains. Toi haute, lui qui noue, ça tenait. Vos voix sont devenues toutes petites. Le ruban reste dans la paume de Chouchou. Je reste un peu. Une mèche à toi, sur le bois. Le tabouret garde une mèche, dans l'ombre jaune.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr"/>
@@ -8687,7 +8687,7 @@
 maman|Vos voix sont devenues toutes petites.
 narrateur|Le ruban reste dans la paume de Chouchou.
 copain|Je reste un peu.
-narrateur|Une poussière reste collée aux cheveux.
+enfant-f|Une mèche à toi, sur le bois.
 narrateur|Le tabouret garde une mèche, dans l'ombre jaune.</t>
         </is>
       </c>
@@ -11160,17 +11160,17 @@
       </c>
       <c r="E55" s="2" t="inlineStr">
         <is>
-          <t>Les talons de Nino sont chauds. Tu as tenu le haut pour moi. Tu nouais le bas. Le carreau sent le soir, tout près. La porte sonnera, demain. Chouchou les pose contre la vitre. Le ruban rouge veille au loquet. Un rai jaune traverse le métal. Le loquet pèse, doré par la rue.</t>
+          <t>Les talons de Nino sont chauds. Tu as tenu le haut pour moi. Tu nouais le bas. Le carreau sent le soir, tout près. La porte sonnera, demain. Je pose le rouge contre la vitre. Le ruban rouge veille au loquet. La rue le dore, un peu. Le loquet pèse, doré par la rue.</t>
         </is>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les talons de Nino sont chauds. Tu as tenu le haut pour moi. Tu nouais le bas. Le carreau sent le soir, tout près. La porte sonnera, demain. Chouchou les pose contre la vitre. Le ruban rouge veille au loquet. Un rai jaune traverse le métal. Le loquet pèse, doré par la rue.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les talons de Nino sont chauds. Tu as tenu le haut pour moi. Tu nouais le bas. Le carreau sent le soir, tout près. La porte sonnera, demain. Je pose le rouge contre la vitre. Le ruban rouge veille au loquet. La rue le dore, un peu. Le loquet pèse, doré par la rue.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les talons de Nino sont chauds. Tu as tenu le haut pour moi. Tu nouais le bas. Le carreau sent le soir, tout près. La porte sonnera, demain. Chouchou les pose contre la vitre. Le ruban rouge veille au loquet. Un rai jaune traverse le métal. Le loquet pèse, doré par la rue.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les talons de Nino sont chauds. Tu as tenu le haut pour moi. Tu nouais le bas. Le carreau sent le soir, tout près. La porte sonnera, demain. Je pose le rouge contre la vitre. Le ruban rouge veille au loquet. La rue le dore, un peu. Le loquet pèse, doré par la rue.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
@@ -11313,9 +11313,9 @@
 copain|Tu nouais le bas.
 maman|Le carreau sent le soir, tout près.
 papa|La porte sonnera, demain.
-narrateur|Chouchou les pose contre la vitre.
+enfant-f|Je pose le rouge contre la vitre.
 narrateur|Le ruban rouge veille au loquet.
-narrateur|Un rai jaune traverse le métal.
+copain|La rue le dore, un peu.
 narrateur|Le loquet pèse, doré par la rue.</t>
         </is>
       </c>
@@ -11532,17 +11532,17 @@
       </c>
       <c r="E57" s="2" t="inlineStr">
         <is>
-          <t>Sur le rebord, deux paires de pieds se touchent. Tu as noué, d'en bas. Tes bras ont tenu le cadre. Chacun a fait sa part, à sa hauteur. Le satin du ruban sèche. Le ruban pose une ombre au plancher. Ça tinte trop, Chouchou. C'est pour ça. Deux paires de pieds se touchent, au rebord.</t>
+          <t>Sur le rebord, deux paires de pieds se touchent. Tu as noué, d'en bas. Tes bras ont tenu le cadre. Chacun a fait sa part, à sa hauteur. Le satin du ruban sèche. Le ruban pose une ombre au plancher. Ça tinte trop, Chouchou. C'est pour ça. Le satin laisse un trait rouge, au rebord.</t>
         </is>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Sur le rebord, deux paires de pieds se touchent. Tu as noué, d'en bas. Tes bras ont tenu le cadre. Chacun a fait sa part, à sa hauteur. Le satin du ruban sèche. Le ruban pose une ombre au plancher. Ça tinte trop, Chouchou. C'est pour ça. Deux paires de pieds se touchent, au rebord.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Sur le rebord, deux paires de pieds se touchent. Tu as noué, d'en bas. Tes bras ont tenu le cadre. Chacun a fait sa part, à sa hauteur. Le satin du ruban sèche. Le ruban pose une ombre au plancher. Ça tinte trop, Chouchou. C'est pour ça. Le satin laisse un trait rouge, au rebord.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Sur le rebord, deux paires de pieds se touchent. Tu as noué, d'en bas. Tes bras ont tenu le cadre. Chacun a fait sa part, à sa hauteur. Le satin du ruban sèche. Le ruban pose une ombre au plancher. Ça tinte trop, Chouchou. C'est pour ça. Deux paires de pieds se touchent, au rebord.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Sur le rebord, deux paires de pieds se touchent. Tu as noué, d'en bas. Tes bras ont tenu le cadre. Chacun a fait sa part, à sa hauteur. Le satin du ruban sèche. Le ruban pose une ombre au plancher. Ça tinte trop, Chouchou. C'est pour ça. Le satin laisse un trait rouge, au rebord.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr"/>
@@ -11688,7 +11688,7 @@
 narrateur|Le ruban pose une ombre au plancher.
 copain|Ça tinte trop, Chouchou.
 enfant-f|C'est pour ça.
-narrateur|Deux paires de pieds se touchent, au rebord.</t>
+narrateur|Le satin laisse un trait rouge, au rebord.</t>
         </is>
       </c>
       <c r="AX57" t="inlineStr">
@@ -13784,17 +13784,17 @@
       </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Sur le tabouret, deux têtes se calment. Nino, tu l'as vue glisser. Oui, tout près de tes mains. Toi haute, lui qui noue, ça tenait. Vos voix sont devenues toutes petites. L'anneau reste dans la paume de Chouchou. Je reste un peu. Une poussière reste collée aux cheveux. Le tabouret sent le bois, sous la lumière.</t>
+          <t>Sur le tabouret, deux têtes se calment. Nino, tu l'as vue glisser. Oui, tout près de tes mains. Toi haute, lui qui noue, ça tenait. Vos voix sont devenues toutes petites. L'anneau reste dans la paume de Chouchou. Je reste un peu. Il a pris ta poussière, Nino. Le tabouret sent le bois, sous la lumière.</t>
         </is>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Sur le tabouret, deux têtes se calment. Nino, tu l'as vue glisser. Oui, tout près de tes mains. Toi haute, lui qui noue, ça tenait. Vos voix sont devenues toutes petites. L'anneau reste dans la paume de Chouchou. Je reste un peu. Une poussière reste collée aux cheveux. Le tabouret sent le bois, sous la lumière.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Sur le tabouret, deux têtes se calment. Nino, tu l'as vue glisser. Oui, tout près de tes mains. Toi haute, lui qui noue, ça tenait. Vos voix sont devenues toutes petites. L'anneau reste dans la paume de Chouchou. Je reste un peu. Il a pris ta poussière, Nino. Le tabouret sent le bois, sous la lumière.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G69" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Sur le tabouret, deux têtes se calment. Nino, tu l'as vue glisser. Oui, tout près de tes mains. Toi haute, lui qui noue, ça tenait. Vos voix sont devenues toutes petites. L'anneau reste dans la paume de Chouchou. Je reste un peu. Une poussière reste collée aux cheveux. Le tabouret sent le bois, sous la lumière.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Sur le tabouret, deux têtes se calment. Nino, tu l'as vue glisser. Oui, tout près de tes mains. Toi haute, lui qui noue, ça tenait. Vos voix sont devenues toutes petites. L'anneau reste dans la paume de Chouchou. Je reste un peu. Il a pris ta poussière, Nino. Le tabouret sent le bois, sous la lumière.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H69" s="2" t="inlineStr"/>
@@ -13939,7 +13939,7 @@
 maman|Vos voix sont devenues toutes petites.
 narrateur|L'anneau reste dans la paume de Chouchou.
 copain|Je reste un peu.
-narrateur|Une poussière reste collée aux cheveux.
+enfant-f|Il a pris ta poussière, Nino.
 narrateur|Le tabouret sent le bois, sous la lumière.</t>
         </is>
       </c>
@@ -16412,17 +16412,17 @@
       </c>
       <c r="E83" s="2" t="inlineStr">
         <is>
-          <t>Les talons de Nino sont chauds. Tu as tenu le haut pour moi. Tu nouais le bas. Le carreau sent le soir, tout près. La porte sonnera, demain. Chouchou les pose contre la vitre. L'anneau de bois veille au loquet. Un rai jaune traverse le métal. Les talons de Nino restent chauds, au loquet.</t>
+          <t>Les talons de Nino sont chauds. Tu as tenu le haut pour moi. Tu nouais le bas. Le carreau sent le soir, tout près. La porte sonnera, demain. Je pose l'anneau contre la vitre. L'anneau de bois veille au loquet. Mes talons sont chauds, là. Les talons de Nino restent chauds, au loquet.</t>
         </is>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les talons de Nino sont chauds. Tu as tenu le haut pour moi. Tu nouais le bas. Le carreau sent le soir, tout près. La porte sonnera, demain. Chouchou les pose contre la vitre. L'anneau de bois veille au loquet. Un rai jaune traverse le métal. Les talons de Nino restent chauds, au loquet.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Les talons de Nino sont chauds. Tu as tenu le haut pour moi. Tu nouais le bas. Le carreau sent le soir, tout près. La porte sonnera, demain. Je pose l'anneau contre la vitre. L'anneau de bois veille au loquet. Mes talons sont chauds, là. Les talons de Nino restent chauds, au loquet.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les talons de Nino sont chauds. Tu as tenu le haut pour moi. Tu nouais le bas. Le carreau sent le soir, tout près. La porte sonnera, demain. Chouchou les pose contre la vitre. L'anneau de bois veille au loquet. Un rai jaune traverse le métal. Les talons de Nino restent chauds, au loquet.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Les talons de Nino sont chauds. Tu as tenu le haut pour moi. Tu nouais le bas. Le carreau sent le soir, tout près. La porte sonnera, demain. Je pose l'anneau contre la vitre. L'anneau de bois veille au loquet. Mes talons sont chauds, là. Les talons de Nino restent chauds, au loquet.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr"/>
@@ -16565,9 +16565,9 @@
 copain|Tu nouais le bas.
 maman|Le carreau sent le soir, tout près.
 papa|La porte sonnera, demain.
-narrateur|Chouchou les pose contre la vitre.
+enfant-f|Je pose l'anneau contre la vitre.
 narrateur|L'anneau de bois veille au loquet.
-narrateur|Un rai jaune traverse le métal.
+copain|Mes talons sont chauds, là.
 narrateur|Les talons de Nino restent chauds, au loquet.</t>
         </is>
       </c>
@@ -17338,7 +17338,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17451,6 +17451,13 @@
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>